<commit_message>
Drop remaining draft file names from the inventory
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZCwLtjiFSY62S3mT8MzgN
</commit_message>
<xml_diff>
--- a/data/analysis_708/01_file_inventory.xlsx
+++ b/data/analysis_708/01_file_inventory.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K312"/>
+  <dimension ref="A1:K308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16587,7 +16587,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Seven-pipleline-comparison-on-Illumina.docx</t>
+          <t>all_species_list_for_simulation_data.docx</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -16606,7 +16606,7 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>1204356</v>
+        <v>69236</v>
       </c>
       <c r="F302" t="inlineStr">
         <is>
@@ -16635,14 +16635,14 @@
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>9ce92ee00935c60e142fb7ff81e87ac7</t>
+          <t>81dc34dbeae77a848c0b46511f7d3b04</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Seven-pipleline-comparison-on-Illumina.md</t>
+          <t>distribution_0.txt</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -16661,7 +16661,7 @@
         </is>
       </c>
       <c r="E303" t="n">
-        <v>37106</v>
+        <v>18408</v>
       </c>
       <c r="F303" t="inlineStr">
         <is>
@@ -16690,14 +16690,14 @@
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>5edc0a7a563fef4c3da3faed94a8c5a9</t>
+          <t>115b7d398d94d9a7c5a8654e2c64b383</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Seven-pipleline-comparison-on-Pacbio.docx</t>
+          <t>distribution_1.txt</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -16716,16 +16716,16 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>1108989</v>
+        <v>18408</v>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>source document</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>source document</t>
+          <t>other</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
@@ -16735,24 +16735,24 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>ground truth / background</t>
+          <t>not a taxon-per-row result table</t>
         </is>
       </c>
       <c r="K304" t="inlineStr">
         <is>
-          <t>3e372b68065c270f2d571dbd9b9cede1</t>
+          <t>8723f0945bffb536a71ba2f4ee2a9658</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Seven-pipleline-comparison-on-Pacbio.md</t>
+          <t>distribution_2.txt</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -16771,7 +16771,7 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>31972</v>
+        <v>18408</v>
       </c>
       <c r="F305" t="inlineStr">
         <is>
@@ -16800,14 +16800,14 @@
       </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>d12a018e5ec746d58cde02774913085c</t>
+          <t>1163cf74c3842911d366dd76c3f5c74d</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>all_species_list_for_simulation_data.docx</t>
+          <t>genome_locations.tsv</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -16826,16 +16826,16 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>69236</v>
+        <v>91912</v>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>source document</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>source document</t>
+          <t>other</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
@@ -16845,24 +16845,24 @@
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>ground truth / background</t>
+          <t>not a taxon-per-row result table</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>81dc34dbeae77a848c0b46511f7d3b04</t>
+          <t>874ae9458b3ffae14b144594dbb143f5</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>distribution_0.txt</t>
+          <t>run_pacbio_sample.sh</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -16881,16 +16881,16 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>18408</v>
+        <v>1225</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>job submission / driver script</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>job submission / driver script</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
@@ -16900,24 +16900,24 @@
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>context only</t>
         </is>
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>not a taxon-per-row result table</t>
+          <t>context only - parameters and versions</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t>115b7d398d94d9a7c5a8654e2c64b383</t>
+          <t>8f195feb50e12aac65b0a91dec83e3cd</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>distribution_1.txt</t>
+          <t>simulate_pacbio.py</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -16936,16 +16936,16 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>18408</v>
+        <v>15400</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>helper script shipped with the run</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>helper script shipped with the run</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
@@ -16955,235 +16955,15 @@
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>context only</t>
         </is>
       </c>
       <c r="J308" t="inlineStr">
         <is>
-          <t>not a taxon-per-row result table</t>
+          <t>context only</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
-        <is>
-          <t>8723f0945bffb536a71ba2f4ee2a9658</t>
-        </is>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="inlineStr">
-        <is>
-          <t>distribution_2.txt</t>
-        </is>
-      </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>n/a (project root)</t>
-        </is>
-      </c>
-      <c r="C309" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D309" t="inlineStr">
-        <is>
-          <t>n/a (pipeline level)</t>
-        </is>
-      </c>
-      <c r="E309" t="n">
-        <v>18408</v>
-      </c>
-      <c r="F309" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G309" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="H309" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I309" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="J309" t="inlineStr">
-        <is>
-          <t>not a taxon-per-row result table</t>
-        </is>
-      </c>
-      <c r="K309" t="inlineStr">
-        <is>
-          <t>1163cf74c3842911d366dd76c3f5c74d</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>genome_locations.tsv</t>
-        </is>
-      </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>n/a (project root)</t>
-        </is>
-      </c>
-      <c r="C310" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D310" t="inlineStr">
-        <is>
-          <t>n/a (pipeline level)</t>
-        </is>
-      </c>
-      <c r="E310" t="n">
-        <v>91912</v>
-      </c>
-      <c r="F310" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G310" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="H310" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I310" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="J310" t="inlineStr">
-        <is>
-          <t>not a taxon-per-row result table</t>
-        </is>
-      </c>
-      <c r="K310" t="inlineStr">
-        <is>
-          <t>874ae9458b3ffae14b144594dbb143f5</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="inlineStr">
-        <is>
-          <t>run_pacbio_sample.sh</t>
-        </is>
-      </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>n/a (project root)</t>
-        </is>
-      </c>
-      <c r="C311" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D311" t="inlineStr">
-        <is>
-          <t>n/a (pipeline level)</t>
-        </is>
-      </c>
-      <c r="E311" t="n">
-        <v>1225</v>
-      </c>
-      <c r="F311" t="inlineStr">
-        <is>
-          <t>job submission / driver script</t>
-        </is>
-      </c>
-      <c r="G311" t="inlineStr">
-        <is>
-          <t>job submission / driver script</t>
-        </is>
-      </c>
-      <c r="H311" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I311" t="inlineStr">
-        <is>
-          <t>context only</t>
-        </is>
-      </c>
-      <c r="J311" t="inlineStr">
-        <is>
-          <t>context only - parameters and versions</t>
-        </is>
-      </c>
-      <c r="K311" t="inlineStr">
-        <is>
-          <t>8f195feb50e12aac65b0a91dec83e3cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>simulate_pacbio.py</t>
-        </is>
-      </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>n/a (project root)</t>
-        </is>
-      </c>
-      <c r="C312" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D312" t="inlineStr">
-        <is>
-          <t>n/a (pipeline level)</t>
-        </is>
-      </c>
-      <c r="E312" t="n">
-        <v>15400</v>
-      </c>
-      <c r="F312" t="inlineStr">
-        <is>
-          <t>helper script shipped with the run</t>
-        </is>
-      </c>
-      <c r="G312" t="inlineStr">
-        <is>
-          <t>helper script shipped with the run</t>
-        </is>
-      </c>
-      <c r="H312" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I312" t="inlineStr">
-        <is>
-          <t>context only</t>
-        </is>
-      </c>
-      <c r="J312" t="inlineStr">
-        <is>
-          <t>context only</t>
-        </is>
-      </c>
-      <c r="K312" t="inlineStr">
         <is>
           <t>36c9e79a0118ab82b730be815df8cac9</t>
         </is>

</xml_diff>